<commit_message>
force test sets to be float
</commit_message>
<xml_diff>
--- a/data/easyData.xlsx
+++ b/data/easyData.xlsx
@@ -96,7 +96,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -128,16 +128,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -146,7 +140,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -459,30 +453,30 @@
   <dimension ref="A1:U10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="33.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="33.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -547,588 +541,588 @@
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1">
         <v>45749.354166666664</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="2">
         <v>5664.75</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="2">
         <v>5665.25</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="2">
         <v>5664.25</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="2">
         <v>5664.75</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="2">
         <v>42.44</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="2">
         <v>-0.87</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="3">
         <v>11</v>
       </c>
-      <c r="I2" s="5">
-        <v>3</v>
-      </c>
-      <c r="J2" s="4">
+      <c r="I2" s="3">
+        <v>3</v>
+      </c>
+      <c r="J2" s="2">
         <v>0.14</v>
       </c>
-      <c r="K2" s="5">
-        <v>3</v>
-      </c>
-      <c r="L2" s="5">
+      <c r="K2" s="3">
+        <v>3</v>
+      </c>
+      <c r="L2" s="3">
         <v>0</v>
       </c>
-      <c r="M2" s="5">
+      <c r="M2" s="3">
         <v>17</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2" s="3">
         <v>15</v>
       </c>
-      <c r="O2" s="5">
-        <v>3</v>
-      </c>
-      <c r="P2" s="5">
-        <v>3</v>
-      </c>
-      <c r="Q2" s="5">
-        <v>3</v>
-      </c>
-      <c r="R2" s="5">
-        <v>1</v>
-      </c>
-      <c r="S2" s="5">
-        <v>3</v>
-      </c>
-      <c r="T2" s="5">
-        <v>3</v>
-      </c>
-      <c r="U2" s="4">
+      <c r="O2" s="3">
+        <v>3</v>
+      </c>
+      <c r="P2" s="3">
+        <v>3</v>
+      </c>
+      <c r="Q2" s="3">
+        <v>3</v>
+      </c>
+      <c r="R2" s="3">
+        <v>1</v>
+      </c>
+      <c r="S2" s="3">
+        <v>3</v>
+      </c>
+      <c r="T2" s="3">
+        <v>3</v>
+      </c>
+      <c r="U2" s="2">
         <v>-0.609</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1">
         <v>45845</v>
       </c>
-      <c r="B3" s="4">
-        <v>5664.75</v>
-      </c>
-      <c r="C3" s="4">
-        <v>5668.5</v>
-      </c>
-      <c r="D3" s="4">
-        <v>5664.5</v>
-      </c>
-      <c r="E3" s="4">
-        <v>5665.75</v>
-      </c>
-      <c r="F3" s="4">
+      <c r="B3" s="2">
+        <v>664.75</v>
+      </c>
+      <c r="C3" s="2">
+        <v>668.5</v>
+      </c>
+      <c r="D3" s="2">
+        <v>664.5</v>
+      </c>
+      <c r="E3" s="2">
+        <v>665.75</v>
+      </c>
+      <c r="F3" s="2">
         <v>64.44</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="2">
         <v>-0.75</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="3">
         <v>11</v>
       </c>
-      <c r="I3" s="5">
-        <v>1</v>
-      </c>
-      <c r="J3" s="4">
+      <c r="I3" s="3">
+        <v>1</v>
+      </c>
+      <c r="J3" s="2">
         <v>0.15</v>
       </c>
-      <c r="K3" s="5">
-        <v>1</v>
-      </c>
-      <c r="L3" s="5">
-        <v>1</v>
-      </c>
-      <c r="M3" s="5">
+      <c r="K3" s="3">
+        <v>1</v>
+      </c>
+      <c r="L3" s="3">
+        <v>1</v>
+      </c>
+      <c r="M3" s="3">
         <v>0</v>
       </c>
-      <c r="N3" s="5">
+      <c r="N3" s="3">
         <v>15</v>
       </c>
-      <c r="O3" s="5">
-        <v>1</v>
-      </c>
-      <c r="P3" s="5">
-        <v>3</v>
-      </c>
-      <c r="Q3" s="5">
-        <v>3</v>
-      </c>
-      <c r="R3" s="5">
-        <v>1</v>
-      </c>
-      <c r="S3" s="5">
-        <v>3</v>
-      </c>
-      <c r="T3" s="5">
-        <v>3</v>
-      </c>
-      <c r="U3" s="4">
+      <c r="O3" s="3">
+        <v>1</v>
+      </c>
+      <c r="P3" s="3">
+        <v>3</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>3</v>
+      </c>
+      <c r="R3" s="3">
+        <v>1</v>
+      </c>
+      <c r="S3" s="3">
+        <v>3</v>
+      </c>
+      <c r="T3" s="3">
+        <v>3</v>
+      </c>
+      <c r="U3" s="2">
         <v>-0.618</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1">
         <v>45749.35428240741</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="2">
         <v>5665.75</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="2">
         <v>5666.5</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="2">
         <v>5665.25</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="2">
         <v>5666.25</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="2">
         <v>65.32</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="2">
         <v>-0.61</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="3">
         <v>9</v>
       </c>
-      <c r="I4" s="5">
-        <v>1</v>
-      </c>
-      <c r="J4" s="4">
+      <c r="I4" s="3">
+        <v>1</v>
+      </c>
+      <c r="J4" s="2">
         <v>0.25</v>
       </c>
-      <c r="K4" s="5">
-        <v>1</v>
-      </c>
-      <c r="L4" s="5">
+      <c r="K4" s="3">
+        <v>1</v>
+      </c>
+      <c r="L4" s="3">
         <v>2</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="3">
         <v>0</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="3">
         <v>13</v>
       </c>
-      <c r="O4" s="5">
-        <v>1</v>
-      </c>
-      <c r="P4" s="5">
-        <v>3</v>
-      </c>
-      <c r="Q4" s="5">
-        <v>3</v>
-      </c>
-      <c r="R4" s="5">
-        <v>1</v>
-      </c>
-      <c r="S4" s="5">
-        <v>1</v>
-      </c>
-      <c r="T4" s="5">
-        <v>3</v>
-      </c>
-      <c r="U4" s="4">
+      <c r="O4" s="3">
+        <v>1</v>
+      </c>
+      <c r="P4" s="3">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="3">
+        <v>3</v>
+      </c>
+      <c r="R4" s="3">
+        <v>1</v>
+      </c>
+      <c r="S4" s="3">
+        <v>1</v>
+      </c>
+      <c r="T4" s="3">
+        <v>3</v>
+      </c>
+      <c r="U4" s="2">
         <v>-0.605</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1">
         <v>45749.35434027778</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="3">
         <v>5666</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="2">
         <v>5667.5</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="2">
         <v>5665.75</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="2">
         <v>5667.25</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="2">
         <v>73.89</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="2">
         <v>-0.41</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="3">
         <v>9</v>
       </c>
-      <c r="I5" s="5">
-        <v>1</v>
-      </c>
-      <c r="J5" s="4">
+      <c r="I5" s="3">
+        <v>1</v>
+      </c>
+      <c r="J5" s="2">
         <v>0.35</v>
       </c>
-      <c r="K5" s="5">
-        <v>1</v>
-      </c>
-      <c r="L5" s="5">
-        <v>3</v>
-      </c>
-      <c r="M5" s="5">
+      <c r="K5" s="3">
+        <v>1</v>
+      </c>
+      <c r="L5" s="3">
+        <v>3</v>
+      </c>
+      <c r="M5" s="3">
         <v>0</v>
       </c>
-      <c r="N5" s="5">
+      <c r="N5" s="3">
         <v>5</v>
       </c>
-      <c r="O5" s="5">
-        <v>1</v>
-      </c>
-      <c r="P5" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q5" s="5">
-        <v>3</v>
-      </c>
-      <c r="R5" s="5">
-        <v>1</v>
-      </c>
-      <c r="S5" s="5">
-        <v>1</v>
-      </c>
-      <c r="T5" s="5">
-        <v>3</v>
-      </c>
-      <c r="U5" s="4">
+      <c r="O5" s="3">
+        <v>1</v>
+      </c>
+      <c r="P5" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="3">
+        <v>3</v>
+      </c>
+      <c r="R5" s="3">
+        <v>1</v>
+      </c>
+      <c r="S5" s="3">
+        <v>1</v>
+      </c>
+      <c r="T5" s="3">
+        <v>3</v>
+      </c>
+      <c r="U5" s="2">
         <v>-0.573</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1">
         <v>45749.35439814815</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="2">
         <v>5667.25</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="2">
         <v>5667.25</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="2">
         <v>5665.75</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="2">
         <v>5666.25</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="2">
         <v>73.89</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="2">
         <v>-0.33</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="3">
         <v>9</v>
       </c>
-      <c r="I6" s="5">
-        <v>1</v>
-      </c>
-      <c r="J6" s="4">
+      <c r="I6" s="3">
+        <v>1</v>
+      </c>
+      <c r="J6" s="2">
         <v>0.36</v>
       </c>
-      <c r="K6" s="5">
-        <v>1</v>
-      </c>
-      <c r="L6" s="5">
+      <c r="K6" s="3">
+        <v>1</v>
+      </c>
+      <c r="L6" s="3">
         <v>4</v>
       </c>
-      <c r="M6" s="5">
+      <c r="M6" s="3">
         <v>0</v>
       </c>
-      <c r="N6" s="5">
+      <c r="N6" s="3">
         <v>5</v>
       </c>
-      <c r="O6" s="5">
-        <v>1</v>
-      </c>
-      <c r="P6" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q6" s="5">
-        <v>3</v>
-      </c>
-      <c r="R6" s="5">
-        <v>1</v>
-      </c>
-      <c r="S6" s="5">
-        <v>1</v>
-      </c>
-      <c r="T6" s="5">
-        <v>3</v>
-      </c>
-      <c r="U6" s="4">
+      <c r="O6" s="3">
+        <v>1</v>
+      </c>
+      <c r="P6" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="3">
+        <v>3</v>
+      </c>
+      <c r="R6" s="3">
+        <v>1</v>
+      </c>
+      <c r="S6" s="3">
+        <v>1</v>
+      </c>
+      <c r="T6" s="3">
+        <v>3</v>
+      </c>
+      <c r="U6" s="2">
         <v>-0.527</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1">
         <v>45749.35445601852</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="2">
         <v>5666.5</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="3">
         <v>5668</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="2">
         <v>5666.5</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="2">
         <v>5667.5</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="2">
         <v>79.25</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="2">
         <v>-0.16</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="3">
         <v>9</v>
       </c>
-      <c r="I7" s="5">
-        <v>1</v>
-      </c>
-      <c r="J7" s="4">
+      <c r="I7" s="3">
+        <v>1</v>
+      </c>
+      <c r="J7" s="2">
         <v>0.4</v>
       </c>
-      <c r="K7" s="5">
-        <v>1</v>
-      </c>
-      <c r="L7" s="5">
+      <c r="K7" s="3">
+        <v>1</v>
+      </c>
+      <c r="L7" s="3">
         <v>5</v>
       </c>
-      <c r="M7" s="5">
+      <c r="M7" s="3">
         <v>0</v>
       </c>
-      <c r="N7" s="5">
+      <c r="N7" s="3">
         <v>5</v>
       </c>
-      <c r="O7" s="5">
-        <v>1</v>
-      </c>
-      <c r="P7" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q7" s="5">
-        <v>3</v>
-      </c>
-      <c r="R7" s="5">
-        <v>1</v>
-      </c>
-      <c r="S7" s="5">
-        <v>1</v>
-      </c>
-      <c r="T7" s="5">
-        <v>3</v>
-      </c>
-      <c r="U7" s="4">
+      <c r="O7" s="3">
+        <v>1</v>
+      </c>
+      <c r="P7" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="3">
+        <v>3</v>
+      </c>
+      <c r="R7" s="3">
+        <v>1</v>
+      </c>
+      <c r="S7" s="3">
+        <v>1</v>
+      </c>
+      <c r="T7" s="3">
+        <v>3</v>
+      </c>
+      <c r="U7" s="2">
         <v>-0.47</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1">
         <v>45749.35451388889</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="2">
         <v>5667.5</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="2">
         <v>5667.5</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="2">
         <v>5664.75</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="3">
         <v>5665</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="2">
         <v>54.19</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="2">
         <v>-0.23</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="3">
         <v>14</v>
       </c>
-      <c r="I8" s="5">
-        <v>1</v>
-      </c>
-      <c r="J8" s="4">
+      <c r="I8" s="3">
+        <v>1</v>
+      </c>
+      <c r="J8" s="2">
         <v>0.16</v>
       </c>
-      <c r="K8" s="5">
-        <v>1</v>
-      </c>
-      <c r="L8" s="5">
+      <c r="K8" s="3">
+        <v>1</v>
+      </c>
+      <c r="L8" s="3">
         <v>6</v>
       </c>
-      <c r="M8" s="5">
+      <c r="M8" s="3">
         <v>0</v>
       </c>
-      <c r="N8" s="5">
+      <c r="N8" s="3">
         <v>2</v>
       </c>
-      <c r="O8" s="5">
-        <v>1</v>
-      </c>
-      <c r="P8" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q8" s="5">
-        <v>3</v>
-      </c>
-      <c r="R8" s="5">
-        <v>1</v>
-      </c>
-      <c r="S8" s="5">
-        <v>1</v>
-      </c>
-      <c r="T8" s="5">
-        <v>3</v>
-      </c>
-      <c r="U8" s="4">
+      <c r="O8" s="3">
+        <v>1</v>
+      </c>
+      <c r="P8" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="3">
+        <v>3</v>
+      </c>
+      <c r="R8" s="3">
+        <v>1</v>
+      </c>
+      <c r="S8" s="3">
+        <v>1</v>
+      </c>
+      <c r="T8" s="3">
+        <v>3</v>
+      </c>
+      <c r="U8" s="2">
         <v>-0.416</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1">
         <v>45749.35457175926</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="2">
         <v>5665.25</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="2">
         <v>5667.5</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="3">
         <v>5665</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="3">
         <v>5667</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="2">
         <v>54.19</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="2">
         <v>-0.12</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="3">
         <v>9</v>
       </c>
-      <c r="I9" s="5">
-        <v>1</v>
-      </c>
-      <c r="J9" s="4">
+      <c r="I9" s="3">
+        <v>1</v>
+      </c>
+      <c r="J9" s="2">
         <v>0.07</v>
       </c>
-      <c r="K9" s="5">
-        <v>1</v>
-      </c>
-      <c r="L9" s="5">
+      <c r="K9" s="3">
+        <v>1</v>
+      </c>
+      <c r="L9" s="3">
         <v>7</v>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="3">
         <v>0</v>
       </c>
-      <c r="N9" s="5">
+      <c r="N9" s="3">
         <v>2</v>
       </c>
-      <c r="O9" s="5">
-        <v>1</v>
-      </c>
-      <c r="P9" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="5">
-        <v>3</v>
-      </c>
-      <c r="R9" s="5">
-        <v>1</v>
-      </c>
-      <c r="S9" s="5">
-        <v>1</v>
-      </c>
-      <c r="T9" s="5">
-        <v>3</v>
-      </c>
-      <c r="U9" s="4">
+      <c r="O9" s="3">
+        <v>1</v>
+      </c>
+      <c r="P9" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="3">
+        <v>3</v>
+      </c>
+      <c r="R9" s="3">
+        <v>1</v>
+      </c>
+      <c r="S9" s="3">
+        <v>1</v>
+      </c>
+      <c r="T9" s="3">
+        <v>3</v>
+      </c>
+      <c r="U9" s="2">
         <v>-0.372</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1">
         <v>45749.354629629626</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="2">
         <v>5666.75</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="2">
         <v>5666.75</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="3">
         <v>5665</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="2">
         <v>5666.75</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="2">
         <v>56.82</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="2">
         <v>-0.05</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="3">
         <v>9</v>
       </c>
-      <c r="I10" s="5">
-        <v>1</v>
-      </c>
-      <c r="J10" s="4">
+      <c r="I10" s="3">
+        <v>1</v>
+      </c>
+      <c r="J10" s="2">
         <v>0.05</v>
       </c>
-      <c r="K10" s="5">
-        <v>3</v>
-      </c>
-      <c r="L10" s="5">
+      <c r="K10" s="3">
+        <v>3</v>
+      </c>
+      <c r="L10" s="3">
         <v>8</v>
       </c>
-      <c r="M10" s="5">
+      <c r="M10" s="3">
         <v>0</v>
       </c>
-      <c r="N10" s="5">
+      <c r="N10" s="3">
         <v>2</v>
       </c>
-      <c r="O10" s="5">
-        <v>1</v>
-      </c>
-      <c r="P10" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q10" s="5">
-        <v>3</v>
-      </c>
-      <c r="R10" s="5">
-        <v>1</v>
-      </c>
-      <c r="S10" s="5">
-        <v>1</v>
-      </c>
-      <c r="T10" s="5">
-        <v>3</v>
-      </c>
-      <c r="U10" s="4">
+      <c r="O10" s="3">
+        <v>1</v>
+      </c>
+      <c r="P10" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="3">
+        <v>3</v>
+      </c>
+      <c r="R10" s="3">
+        <v>1</v>
+      </c>
+      <c r="S10" s="3">
+        <v>1</v>
+      </c>
+      <c r="T10" s="3">
+        <v>3</v>
+      </c>
+      <c r="U10" s="2">
         <v>-0.336</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Still a work in progress
</commit_message>
<xml_diff>
--- a/data/easyData.xlsx
+++ b/data/easyData.xlsx
@@ -608,19 +608,19 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1">
-        <v>45863</v>
+        <v>45749.35422453703</v>
       </c>
       <c r="B3" s="2">
-        <v>664.75</v>
+        <v>5664.75</v>
       </c>
       <c r="C3" s="2">
-        <v>668.5</v>
+        <v>5668.5</v>
       </c>
       <c r="D3" s="2">
-        <v>664.5</v>
+        <v>5664.5</v>
       </c>
       <c r="E3" s="2">
-        <v>665.75</v>
+        <v>5665.75</v>
       </c>
       <c r="F3" s="2">
         <v>64.44</v>
@@ -933,7 +933,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1">
-        <v>45750</v>
+        <v>45749.35451388889</v>
       </c>
       <c r="B8" s="2">
         <v>5667.5</v>

</xml_diff>